<commit_message>
Add curative recommendations: turn the defect list into an actionable worklist
Each defect now carries a concrete, plain-language curative action (standard
title-curative steps, not a conclusion). src/databossx/curative.py maps defect
category + detail patterns to a recommendation -- e.g. an over-conveyance,
chain-of-title break, 8/8 shortfall, or unreadable evidence each get a specific
next step. Surfaced as a "Curative Action" column in the Defects sheet, the PDF
defect table, and the dashboard.

Tests: +5. Full suite: 199 passed, 7 skipped. flake8 clean. Refreshed synthetic
sample outputs include the curative column.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014JmLn9nD8x9Yc5Jjdgyqw6
</commit_message>
<xml_diff>
--- a/examples/sample_output/GOLDEN-DEMO/DataBossX_Report.xlsx
+++ b/examples/sample_output/GOLDEN-DEMO/DataBossX_Report.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-18 16:38:09 UTC</t>
+          <t>2026-07-18 16:48:10 UTC</t>
         </is>
       </c>
     </row>
@@ -2405,20 +2405,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="54" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Defects &amp; missing evidence -- resolve before release</t>
+          <t>Defects &amp; curative worklist -- resolve before release</t>
         </is>
       </c>
     </row>
@@ -2445,6 +2446,11 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
+          <t>Curative Action</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
@@ -2472,6 +2478,11 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
+          <t>Over-conveyance: the grantor purported to convey more than the record shows they held. Confirm the grantor's actual interest and whether a prior conveyance or reservation is missing from the chain before relying on any downstream interest.</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
           <t>runsheet chain</t>
         </is>
       </c>
@@ -2499,6 +2510,11 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
+          <t>Locate the instrument (or its recording data) that links this document across the OGL register and the runsheet. If none exists, document the gap and obtain the missing conveyance.</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
           <t>OGL/runsheet cross-ref</t>
         </is>
       </c>
@@ -2526,6 +2542,11 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
+          <t>Locate the instrument (or its recording data) that links this document across the OGL register and the runsheet. If none exists, document the gap and obtain the missing conveyance.</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
           <t>OGL/runsheet cross-ref</t>
         </is>
       </c>
@@ -2553,13 +2574,18 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
+          <t>Reconcile the mineral estate to a full 8/8: find the instrument(s) that convey the missing or excess undivided interest, or confirm and record an outstanding unleased interest.</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
           <t>division of interest</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2742,7 +2768,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>9591ac7a23c63b0479e7b1a84d3226cf942c40ae8a10e6da082c538852edab32</t>
+          <t>4cf7a3ce55455c4983b7b5e39acf3ab7068b1191aa65353fd40fb2827ce44b07</t>
         </is>
       </c>
       <c r="D7" t="n">

</xml_diff>